<commit_message>
chore: atualiza gitignore e remove dados sensiveis do rastreamento
</commit_message>
<xml_diff>
--- a/respostas_forms_rotina.xlsx
+++ b/respostas_forms_rotina.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\1_Arquivos\Trabalho\UNIVESP\sistema-preditivo-evasao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{607B0195-1FE7-456F-8489-FAACF53F6BB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8629992-224D-40C6-94CA-9404718178A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -365,22 +365,6 @@
       </font>
     </dxf>
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF5B3F86"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF5B3F86"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF5B3F86"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF5B3F86"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF8F9FA"/>
@@ -404,13 +388,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF5B3F86"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF5B3F86"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF5B3F86"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF5B3F86"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
     <tableStyle name="Respostas ao formulário 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="13"/>
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="firstRowStripe" dxfId="15"/>
-      <tableStyleElement type="secondRowStripe" dxfId="14"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="secondRowStripe" dxfId="13"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -429,18 +429,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:J38" headerRowDxfId="2" dataDxfId="0" totalsRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:J38" headerRowDxfId="12" dataDxfId="11" totalsRowDxfId="10">
   <tableColumns count="10">
-    <tableColumn id="12" xr3:uid="{0B362407-35DA-4FD3-8998-92CC50DFCEAD}" name="Código SGDE" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="2)  Qual é a sua situação de trabalho atual? " dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="3)  Qual é a sua carga horária de trabalho diária? " dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="4)  Como você avalia o esforço físico exigido no seu trabalho? " dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="5)  Como é a sua rotina de deslocamento para a escola? " dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="6)  Em média, quantas horas de sono você consegue ter por noite durante a semana?  " dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="7)  Sobre a sua alimentação antes de chegar à escola: " dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="8)  O seu meio de transporte para a escola é sujeito a atrasos frequentes ou problemas (ex: ônibus rural que quebra, carona incerta, ônibus de linha atrasado)? " dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="9)  Qual o seu principal objetivo ao concluir o Ensino Médio? " dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="10) Qual o horário que você sai do seu trabalho?" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{0B362407-35DA-4FD3-8998-92CC50DFCEAD}" name="Código SGDE" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="2)  Qual é a sua situação de trabalho atual? " dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="3)  Qual é a sua carga horária de trabalho diária? " dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="4)  Como você avalia o esforço físico exigido no seu trabalho? " dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="5)  Como é a sua rotina de deslocamento para a escola? " dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="6)  Em média, quantas horas de sono você consegue ter por noite durante a semana?  " dataDxfId="4"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="7)  Sobre a sua alimentação antes de chegar à escola: " dataDxfId="3"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="8)  O seu meio de transporte para a escola é sujeito a atrasos frequentes ou problemas (ex: ônibus rural que quebra, carona incerta, ônibus de linha atrasado)? " dataDxfId="2"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="9)  Qual o seu principal objetivo ao concluir o Ensino Médio? " dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="10) Qual o horário que você sai do seu trabalho?" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>